<commit_message>
docs(chp3): streamline Research Approach, hypotheses, partitioning and validity per author directives
</commit_message>
<xml_diff>
--- a/results/methodology-tables.xlsx
+++ b/results/methodology-tables.xlsx
@@ -588,7 +588,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="38" customHeight="1">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Phase 1</t>
@@ -622,7 +622,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="38" customHeight="1">
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Phase 2</t>
@@ -640,7 +640,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>• Baseline Control: Formulate diurnal persistence benchmark (Vol_t = Vol_{t-24}, non-parametric MASE = 1.000).
+          <t>• Baseline Control: Formulate diurnal persistence benchmark (Vol_hat_t = Vol_{t-24}, non-parametric MASE = 1.000).
 • Model 1 (Deterministic): Implement operational flight schedule convolution based on ACRP Report 40 passenger arrival curves.
 • Model 2 (Machine Learning): Train decision-tree regressor on convolved schedules and 24 BTS OTP operational features.
 • Model 3 (Dynamic Hybrid): Construct two-stage hybrid coupling recurring schedule cycles with live 1-step floor error feedback (e_{t-1} = y_{t-1} - y_hat_{t-1}).</t>
@@ -654,7 +654,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="38" customHeight="1">
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Phase 3</t>
@@ -686,7 +686,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="38" customHeight="1">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Phase 4</t>
@@ -786,7 +786,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="38" customHeight="1">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Phase 1: Ingestion &amp; ETL</t>
@@ -818,7 +818,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="38" customHeight="1">
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Phase 1: Ingestion &amp; ETL</t>
@@ -850,7 +850,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="38" customHeight="1">
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Phase 1: Ingestion &amp; ETL</t>
@@ -882,7 +882,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="38" customHeight="1">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Phase 1: Ingestion &amp; ETL</t>
@@ -914,7 +914,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="38" customHeight="1">
+    <row r="9" ht="36" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Phase 1: Ingestion &amp; ETL</t>
@@ -946,7 +946,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="38" customHeight="1">
+    <row r="10" ht="36" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Phase 1: Ingestion &amp; ETL</t>
@@ -978,7 +978,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="38" customHeight="1">
+    <row r="11" ht="36" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Phase 1: Ingestion &amp; ETL</t>
@@ -1010,7 +1010,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="38" customHeight="1">
+    <row r="12" ht="36" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Phase 1: Ingestion &amp; ETL</t>
@@ -1042,7 +1042,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="38" customHeight="1">
+    <row r="13" ht="36" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Phase 2: Model Development</t>
@@ -1074,7 +1074,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="38" customHeight="1">
+    <row r="14" ht="36" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Phase 2: Model Development</t>
@@ -1106,7 +1106,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="38" customHeight="1">
+    <row r="15" ht="36" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Phase 2: Model Development</t>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Conformed feature store (Candidate B partition); LightGBM / Scikit-learn regressors.</t>
+          <t>Conformed feature store; LightGBM / Scikit-learn regressors.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -1138,7 +1138,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="38" customHeight="1">
+    <row r="16" ht="36" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Phase 2: Model Development</t>
@@ -1170,7 +1170,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="38" customHeight="1">
+    <row r="17" ht="36" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Phase 3: Evaluation</t>
@@ -1202,7 +1202,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="38" customHeight="1">
+    <row r="18" ht="36" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Phase 3: Evaluation</t>
@@ -1234,7 +1234,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="38" customHeight="1">
+    <row r="19" ht="36" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Phase 3: Evaluation</t>
@@ -1266,7 +1266,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="38" customHeight="1">
+    <row r="20" ht="36" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Phase 3: Evaluation</t>
@@ -1298,7 +1298,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="38" customHeight="1">
+    <row r="21" ht="36" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Phase 3: Evaluation</t>
@@ -1330,7 +1330,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="38" customHeight="1">
+    <row r="22" ht="36" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Phase 4: Interpretation</t>
@@ -1358,11 +1358,11 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Formal academic validation of H1, H1a, H1b, and H1c.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="38" customHeight="1">
+          <t>Formal academic validation of H1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Phase 4: Interpretation</t>
@@ -1394,7 +1394,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="38" customHeight="1">
+    <row r="24" ht="36" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Phase 4: Interpretation</t>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="38" customHeight="1">
+    <row r="25" ht="36" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Phase 4: Interpretation</t>
@@ -1469,31 +1469,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table 3.2: Longitudinal Dataset Partitioning and Validation Protocol</t>
+          <t>Table A.2: Longitudinal Dataset Partitioning and Validation Protocol</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Candidate B Partitioning Design Across 44 Continuous Calendar Months (May 1, 2022 – December 31, 2025) with Operational Purge Buffers</t>
+          <t>Partitioning Design Across 44 Continuous Calendar Months (May 1, 2022 – December 31, 2025)</t>
         </is>
       </c>
     </row>
@@ -1538,13 +1537,8 @@
           <t>Methodological Function &amp; Validation Role</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Purge Buffer &amp; Integrity Protocol</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="38" customHeight="1">
+    </row>
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Training Window</t>
@@ -1582,91 +1576,81 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Calibrate ACRP Report 40 flight schedule convolution baseline; train decision-tree regressors on BTS OTP operational features; establish initial hybrid Stage 1 cycles.</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>Established post-pandemic (May 1, 2022); vacatur of transit mask mandate and load factor rebound to 84.7% baseline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="38" customHeight="1">
+          <t>Calibrate flight schedule convolution baseline; train decision-tree regressors on BTS OTP operational features; establish initial hybrid Stage 1 cycles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Operational Purge Buffer 1</t>
+          <t>Validation Window</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Temporal Separation Interval</t>
+          <t>Hyperparameter Tuning &amp; Optimization</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Jan 1, 2024 – Jan 7, 2024</t>
+          <t>Jan 8, 2024 – Dec 24, 2024</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>7 Days</t>
+          <t>11.8 Months</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Excluded</t>
+          <t>3,293</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Excluded</t>
+          <t>72,723</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Purge Interval</t>
+          <t>9 Airports / 12 Complexes</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Quarantine multi-day holiday travel delay cascades and severe winter weather disruptions from bleeding across development partition boundaries.</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="inlineStr">
-        <is>
-          <t>Strict 7-day purge buffer eliminates temporal autocorrelation and lookahead contamination between training and validation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="38" customHeight="1">
+          <t>Strictly reserved for hyperparameter tuning (tree depth, minimum leaf size, learning rate), cross-validation, and error innovation loop gain calibration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Validation Window</t>
+          <t>Out-of-Time Holdout Window</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Hyperparameter Tuning &amp; Optimization</t>
+          <t>Blind Empirical Holdout Evaluation</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Jan 8, 2024 – Dec 24, 2024</t>
+          <t>Jan 1, 2025 – Dec 31, 2025</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>11.8 Months</t>
+          <t>12.0 Months</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>3,293</t>
+          <t>3,222</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>72,723</t>
+          <t>72,053</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1676,153 +1660,49 @@
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Strictly reserved for hyperparameter tuning (tree depth, minimum leaf size, learning rate), cross-validation, and error innovation loop gain calibration.</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>Prevents model snooping and hyperparameter overfit; models frozen prior to deployment on out-of-time holdout.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Operational Purge Buffer 2</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Temporal Separation Interval</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Dec 25, 2024 – Dec 31, 2024</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>7 Days</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>Excluded</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>Excluded</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Purge Interval</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>Quarantine peak winter holiday irregular operations (IROPS) and cascading cancellation shocks from leaking into the blind out-of-time evaluation year.</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr">
-        <is>
-          <t>Strict 7-day operational purge buffer guarantees pristine out-of-time evaluation boundary.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="38" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Out-of-Time Holdout Window</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Blind Empirical Holdout Evaluation</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Jan 1, 2025 – Dec 31, 2025</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>12.0 Months</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>3,222</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>72,053</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
+          <t>Certified out-of-time evaluation suite. Benchmarks all candidate architectures across Robustness (routine operations), Resilience (severe IROPS), and Generalizability (zero-shot transfer).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Total Longitudinal Dataset</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Full Continuous Study Sequence</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>May 1, 2022 – Dec 31, 2025</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>44.0 Months</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>22,491</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>267,623</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>9 Airports / 12 Complexes</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Certified out-of-time evaluation suite. Benchmarks all candidate architectures across Robustness (routine operations), Resilience (severe IROPS), and Generalizability (zero-shot transfer).</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>Completely blind, untouched test partition; foundation for certified hypothesis testing (H1) and Diebold-Mariano evaluation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="38" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>Total Longitudinal Dataset</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Full Continuous Study Sequence</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>May 1, 2022 – Dec 31, 2025</t>
-        </is>
-      </c>
-      <c r="D10" s="11" t="inlineStr">
-        <is>
-          <t>44.0 Months</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>22,491</t>
-        </is>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
-        <is>
-          <t>267,623</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="inlineStr">
-        <is>
-          <t>9 Airports / 12 Complexes</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="H8" s="10" t="inlineStr">
         <is>
           <t>Comprehensive longitudinal empirical foundation tracking carrier-exclusive terminal screening complexes across all four structural airport archetypes.</t>
-        </is>
-      </c>
-      <c r="I10" s="10" t="inlineStr">
-        <is>
-          <t>100% non-null record audit; zero orphan foreign keys; complete referential integrity across 2.70B screened passengers.</t>
         </is>
       </c>
     </row>
@@ -1853,7 +1733,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Table 3.3: Primary Authorized Secondary Data Sources and Repository Census</t>
+          <t>Table A.3: Primary Authorized Secondary Data Sources and Repository Census</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1786,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="38" customHeight="1">
+    <row r="5" ht="36" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>TSA FOIA Checkpoint Screening Logs</t>
@@ -1950,7 +1830,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="38" customHeight="1">
+    <row r="6" ht="36" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>BTS On-Time Flight Performance (OTP)</t>
@@ -1994,7 +1874,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="38" customHeight="1">
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>BTS Form 41 Schedule T-100 Segment Data</t>
@@ -2038,7 +1918,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="38" customHeight="1">
+    <row r="8" ht="36" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>BTS DB1B / DB1C Ticket Surveys</t>
@@ -2082,7 +1962,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="38" customHeight="1">
+    <row r="9" ht="36" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Total Integrated Feature Warehouse</t>

</xml_diff>